<commit_message>
Store Checkers article keys as numbers so SUMIF matches cleanly
Both sides were text, which risks SUMIF coercing the criterion and
silently returning zeros.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014G7TrxwxBYrrbPWFRWRcNS
</commit_message>
<xml_diff>
--- a/prep/checkers/Creative Beverages - Checkers read.xlsx
+++ b/prep/checkers/Creative Beverages - Checkers read.xlsx
@@ -1989,10 +1989,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>10755051</t>
-        </is>
+      <c r="B5" s="20" t="n">
+        <v>10755051</v>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
@@ -2045,10 +2043,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>10755051</t>
-        </is>
+      <c r="B6" s="20" t="n">
+        <v>10755051</v>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
@@ -2101,10 +2097,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>10755051</t>
-        </is>
+      <c r="B7" s="20" t="n">
+        <v>10755051</v>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
@@ -2157,10 +2151,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>10755051</t>
-        </is>
+      <c r="B8" s="20" t="n">
+        <v>10755051</v>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
@@ -2213,10 +2205,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>10969386</t>
-        </is>
+      <c r="B9" s="20" t="n">
+        <v>10969386</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -2269,10 +2259,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>10969386</t>
-        </is>
+      <c r="B10" s="20" t="n">
+        <v>10969386</v>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
@@ -2325,10 +2313,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>10969386</t>
-        </is>
+      <c r="B11" s="20" t="n">
+        <v>10969386</v>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
@@ -2381,10 +2367,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>10711455</t>
-        </is>
+      <c r="B12" s="20" t="n">
+        <v>10711455</v>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
@@ -2437,10 +2421,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>10711455</t>
-        </is>
+      <c r="B13" s="20" t="n">
+        <v>10711455</v>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
@@ -2493,10 +2475,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>10711455</t>
-        </is>
+      <c r="B14" s="20" t="n">
+        <v>10711455</v>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
@@ -2549,10 +2529,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B15" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
@@ -2605,10 +2583,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B16" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
@@ -2661,10 +2637,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B17" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
@@ -2717,10 +2691,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B18" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
@@ -2773,10 +2745,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B19" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C19" s="20" t="inlineStr">
         <is>
@@ -2829,10 +2799,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B20" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
@@ -2885,10 +2853,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>10483608</t>
-        </is>
+      <c r="B21" s="20" t="n">
+        <v>10483608</v>
       </c>
       <c r="C21" s="20" t="inlineStr">
         <is>
@@ -2941,10 +2907,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
-        <is>
-          <t>10483608</t>
-        </is>
+      <c r="B22" s="20" t="n">
+        <v>10483608</v>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
@@ -2997,10 +2961,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>10483608</t>
-        </is>
+      <c r="B23" s="20" t="n">
+        <v>10483608</v>
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
@@ -3053,10 +3015,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
-        <is>
-          <t>10521085</t>
-        </is>
+      <c r="B24" s="20" t="n">
+        <v>10521085</v>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
@@ -3109,10 +3069,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>10521085</t>
-        </is>
+      <c r="B25" s="20" t="n">
+        <v>10521085</v>
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
@@ -3165,10 +3123,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>10521085</t>
-        </is>
+      <c r="B26" s="20" t="n">
+        <v>10521085</v>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
@@ -3221,10 +3177,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
-        <is>
-          <t>10532818</t>
-        </is>
+      <c r="B27" s="20" t="n">
+        <v>10532818</v>
       </c>
       <c r="C27" s="20" t="inlineStr">
         <is>
@@ -3277,10 +3231,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
-        <is>
-          <t>10532818</t>
-        </is>
+      <c r="B28" s="20" t="n">
+        <v>10532818</v>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
@@ -3333,10 +3285,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
-        <is>
-          <t>10532818</t>
-        </is>
+      <c r="B29" s="20" t="n">
+        <v>10532818</v>
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
@@ -3389,10 +3339,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
-        <is>
-          <t>10532819</t>
-        </is>
+      <c r="B30" s="20" t="n">
+        <v>10532819</v>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
@@ -3445,10 +3393,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
-        <is>
-          <t>10532819</t>
-        </is>
+      <c r="B31" s="20" t="n">
+        <v>10532819</v>
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
@@ -3501,10 +3447,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
-        <is>
-          <t>10532819</t>
-        </is>
+      <c r="B32" s="20" t="n">
+        <v>10532819</v>
       </c>
       <c r="C32" s="20" t="inlineStr">
         <is>
@@ -3557,10 +3501,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
-        <is>
-          <t>10697191</t>
-        </is>
+      <c r="B33" s="20" t="n">
+        <v>10697191</v>
       </c>
       <c r="C33" s="20" t="inlineStr">
         <is>
@@ -3613,10 +3555,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
-        <is>
-          <t>10697191</t>
-        </is>
+      <c r="B34" s="20" t="n">
+        <v>10697191</v>
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
@@ -3669,10 +3609,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
-        <is>
-          <t>10697191</t>
-        </is>
+      <c r="B35" s="20" t="n">
+        <v>10697191</v>
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
@@ -3725,10 +3663,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
-        <is>
-          <t>10810779</t>
-        </is>
+      <c r="B36" s="20" t="n">
+        <v>10810779</v>
       </c>
       <c r="C36" s="20" t="inlineStr">
         <is>
@@ -3781,10 +3717,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
-        <is>
-          <t>10810779</t>
-        </is>
+      <c r="B37" s="20" t="n">
+        <v>10810779</v>
       </c>
       <c r="C37" s="20" t="inlineStr">
         <is>
@@ -3837,10 +3771,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
-        <is>
-          <t>10810779</t>
-        </is>
+      <c r="B38" s="20" t="n">
+        <v>10810779</v>
       </c>
       <c r="C38" s="20" t="inlineStr">
         <is>
@@ -3893,10 +3825,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B39" s="20" t="inlineStr">
-        <is>
-          <t>10810780</t>
-        </is>
+      <c r="B39" s="20" t="n">
+        <v>10810780</v>
       </c>
       <c r="C39" s="20" t="inlineStr">
         <is>
@@ -3949,10 +3879,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B40" s="20" t="inlineStr">
-        <is>
-          <t>10810780</t>
-        </is>
+      <c r="B40" s="20" t="n">
+        <v>10810780</v>
       </c>
       <c r="C40" s="20" t="inlineStr">
         <is>
@@ -4005,10 +3933,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
-        <is>
-          <t>10810780</t>
-        </is>
+      <c r="B41" s="20" t="n">
+        <v>10810780</v>
       </c>
       <c r="C41" s="20" t="inlineStr">
         <is>
@@ -4061,10 +3987,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B42" s="20" t="inlineStr">
-        <is>
-          <t>10810782</t>
-        </is>
+      <c r="B42" s="20" t="n">
+        <v>10810782</v>
       </c>
       <c r="C42" s="20" t="inlineStr">
         <is>
@@ -4117,10 +4041,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
-        <is>
-          <t>10810782</t>
-        </is>
+      <c r="B43" s="20" t="n">
+        <v>10810782</v>
       </c>
       <c r="C43" s="20" t="inlineStr">
         <is>
@@ -4173,10 +4095,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B44" s="20" t="inlineStr">
-        <is>
-          <t>10810782</t>
-        </is>
+      <c r="B44" s="20" t="n">
+        <v>10810782</v>
       </c>
       <c r="C44" s="20" t="inlineStr">
         <is>
@@ -4229,10 +4149,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
-        <is>
-          <t>10935004</t>
-        </is>
+      <c r="B45" s="20" t="n">
+        <v>10935004</v>
       </c>
       <c r="C45" s="20" t="inlineStr">
         <is>
@@ -4285,10 +4203,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B46" s="20" t="inlineStr">
-        <is>
-          <t>10935004</t>
-        </is>
+      <c r="B46" s="20" t="n">
+        <v>10935004</v>
       </c>
       <c r="C46" s="20" t="inlineStr">
         <is>
@@ -4341,10 +4257,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
-        <is>
-          <t>10935004</t>
-        </is>
+      <c r="B47" s="20" t="n">
+        <v>10935004</v>
       </c>
       <c r="C47" s="20" t="inlineStr">
         <is>
@@ -4397,10 +4311,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B48" s="20" t="inlineStr">
-        <is>
-          <t>10908314</t>
-        </is>
+      <c r="B48" s="20" t="n">
+        <v>10908314</v>
       </c>
       <c r="C48" s="20" t="inlineStr">
         <is>
@@ -4453,10 +4365,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B49" s="20" t="inlineStr">
-        <is>
-          <t>10908314</t>
-        </is>
+      <c r="B49" s="20" t="n">
+        <v>10908314</v>
       </c>
       <c r="C49" s="20" t="inlineStr">
         <is>
@@ -4509,10 +4419,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B50" s="20" t="inlineStr">
-        <is>
-          <t>10908314</t>
-        </is>
+      <c r="B50" s="20" t="n">
+        <v>10908314</v>
       </c>
       <c r="C50" s="20" t="inlineStr">
         <is>
@@ -4565,10 +4473,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B51" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B51" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C51" s="20" t="inlineStr">
         <is>
@@ -4621,10 +4527,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B52" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B52" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C52" s="20" t="inlineStr">
         <is>
@@ -4677,10 +4581,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B53" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B53" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C53" s="20" t="inlineStr">
         <is>
@@ -4733,10 +4635,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B54" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B54" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C54" s="20" t="inlineStr">
         <is>
@@ -4789,10 +4689,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B55" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C55" s="20" t="inlineStr">
         <is>
@@ -4845,10 +4743,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B56" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B56" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C56" s="20" t="inlineStr">
         <is>
@@ -4901,10 +4797,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B57" s="20" t="inlineStr">
-        <is>
-          <t>10908316</t>
-        </is>
+      <c r="B57" s="20" t="n">
+        <v>10908316</v>
       </c>
       <c r="C57" s="20" t="inlineStr">
         <is>
@@ -4957,10 +4851,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B58" s="20" t="inlineStr">
-        <is>
-          <t>10908316</t>
-        </is>
+      <c r="B58" s="20" t="n">
+        <v>10908316</v>
       </c>
       <c r="C58" s="20" t="inlineStr">
         <is>
@@ -5013,10 +4905,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B59" s="20" t="inlineStr">
-        <is>
-          <t>10908316</t>
-        </is>
+      <c r="B59" s="20" t="n">
+        <v>10908316</v>
       </c>
       <c r="C59" s="20" t="inlineStr">
         <is>
@@ -5069,10 +4959,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B60" s="20" t="inlineStr">
-        <is>
-          <t>10615602</t>
-        </is>
+      <c r="B60" s="20" t="n">
+        <v>10615602</v>
       </c>
       <c r="C60" s="20" t="inlineStr">
         <is>
@@ -5125,10 +5013,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B61" s="20" t="inlineStr">
-        <is>
-          <t>10615602</t>
-        </is>
+      <c r="B61" s="20" t="n">
+        <v>10615602</v>
       </c>
       <c r="C61" s="20" t="inlineStr">
         <is>
@@ -5181,10 +5067,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B62" s="20" t="inlineStr">
-        <is>
-          <t>10615602</t>
-        </is>
+      <c r="B62" s="20" t="n">
+        <v>10615602</v>
       </c>
       <c r="C62" s="20" t="inlineStr">
         <is>
@@ -5237,10 +5121,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B63" s="20" t="inlineStr">
-        <is>
-          <t>10615602</t>
-        </is>
+      <c r="B63" s="20" t="n">
+        <v>10615602</v>
       </c>
       <c r="C63" s="20" t="inlineStr">
         <is>
@@ -5293,10 +5175,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B64" s="20" t="inlineStr">
-        <is>
-          <t>10615603</t>
-        </is>
+      <c r="B64" s="20" t="n">
+        <v>10615603</v>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
@@ -5349,10 +5229,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B65" s="20" t="inlineStr">
-        <is>
-          <t>10615603</t>
-        </is>
+      <c r="B65" s="20" t="n">
+        <v>10615603</v>
       </c>
       <c r="C65" s="20" t="inlineStr">
         <is>
@@ -5405,10 +5283,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B66" s="20" t="inlineStr">
-        <is>
-          <t>10615603</t>
-        </is>
+      <c r="B66" s="20" t="n">
+        <v>10615603</v>
       </c>
       <c r="C66" s="20" t="inlineStr">
         <is>
@@ -5461,10 +5337,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B67" s="20" t="inlineStr">
-        <is>
-          <t>10615603</t>
-        </is>
+      <c r="B67" s="20" t="n">
+        <v>10615603</v>
       </c>
       <c r="C67" s="20" t="inlineStr">
         <is>
@@ -5517,10 +5391,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B68" s="20" t="inlineStr">
-        <is>
-          <t>10787565</t>
-        </is>
+      <c r="B68" s="20" t="n">
+        <v>10787565</v>
       </c>
       <c r="C68" s="20" t="inlineStr">
         <is>
@@ -5573,10 +5445,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B69" s="20" t="inlineStr">
-        <is>
-          <t>10787565</t>
-        </is>
+      <c r="B69" s="20" t="n">
+        <v>10787565</v>
       </c>
       <c r="C69" s="20" t="inlineStr">
         <is>
@@ -5629,10 +5499,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B70" s="20" t="inlineStr">
-        <is>
-          <t>10787565</t>
-        </is>
+      <c r="B70" s="20" t="n">
+        <v>10787565</v>
       </c>
       <c r="C70" s="20" t="inlineStr">
         <is>
@@ -5685,10 +5553,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B71" s="20" t="inlineStr">
-        <is>
-          <t>10842437</t>
-        </is>
+      <c r="B71" s="20" t="n">
+        <v>10842437</v>
       </c>
       <c r="C71" s="20" t="inlineStr">
         <is>
@@ -5741,10 +5607,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B72" s="20" t="inlineStr">
-        <is>
-          <t>10842437</t>
-        </is>
+      <c r="B72" s="20" t="n">
+        <v>10842437</v>
       </c>
       <c r="C72" s="20" t="inlineStr">
         <is>
@@ -5797,10 +5661,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B73" s="20" t="inlineStr">
-        <is>
-          <t>10842437</t>
-        </is>
+      <c r="B73" s="20" t="n">
+        <v>10842437</v>
       </c>
       <c r="C73" s="20" t="inlineStr">
         <is>
@@ -5853,10 +5715,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B74" s="20" t="inlineStr">
-        <is>
-          <t>10864669</t>
-        </is>
+      <c r="B74" s="20" t="n">
+        <v>10864669</v>
       </c>
       <c r="C74" s="20" t="inlineStr">
         <is>
@@ -5909,10 +5769,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B75" s="20" t="inlineStr">
-        <is>
-          <t>10864669</t>
-        </is>
+      <c r="B75" s="20" t="n">
+        <v>10864669</v>
       </c>
       <c r="C75" s="20" t="inlineStr">
         <is>
@@ -5965,10 +5823,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B76" s="20" t="inlineStr">
-        <is>
-          <t>10864669</t>
-        </is>
+      <c r="B76" s="20" t="n">
+        <v>10864669</v>
       </c>
       <c r="C76" s="20" t="inlineStr">
         <is>
@@ -6021,10 +5877,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B77" s="20" t="inlineStr">
-        <is>
-          <t>10864670</t>
-        </is>
+      <c r="B77" s="20" t="n">
+        <v>10864670</v>
       </c>
       <c r="C77" s="20" t="inlineStr">
         <is>
@@ -6077,10 +5931,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B78" s="20" t="inlineStr">
-        <is>
-          <t>10864670</t>
-        </is>
+      <c r="B78" s="20" t="n">
+        <v>10864670</v>
       </c>
       <c r="C78" s="20" t="inlineStr">
         <is>
@@ -6133,10 +5985,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B79" s="20" t="inlineStr">
-        <is>
-          <t>10864670</t>
-        </is>
+      <c r="B79" s="20" t="n">
+        <v>10864670</v>
       </c>
       <c r="C79" s="20" t="inlineStr">
         <is>
@@ -6189,10 +6039,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B80" s="20" t="inlineStr">
-        <is>
-          <t>10866366</t>
-        </is>
+      <c r="B80" s="20" t="n">
+        <v>10866366</v>
       </c>
       <c r="C80" s="20" t="inlineStr">
         <is>
@@ -6245,10 +6093,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B81" s="20" t="inlineStr">
-        <is>
-          <t>10937405</t>
-        </is>
+      <c r="B81" s="20" t="n">
+        <v>10937405</v>
       </c>
       <c r="C81" s="20" t="inlineStr">
         <is>
@@ -6301,10 +6147,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B82" s="20" t="inlineStr">
-        <is>
-          <t>10937405</t>
-        </is>
+      <c r="B82" s="20" t="n">
+        <v>10937405</v>
       </c>
       <c r="C82" s="20" t="inlineStr">
         <is>
@@ -6357,10 +6201,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B83" s="20" t="inlineStr">
-        <is>
-          <t>10937405</t>
-        </is>
+      <c r="B83" s="20" t="n">
+        <v>10937405</v>
       </c>
       <c r="C83" s="20" t="inlineStr">
         <is>
@@ -6413,10 +6255,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B84" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B84" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C84" s="20" t="inlineStr">
         <is>
@@ -6469,10 +6309,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B85" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B85" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C85" s="20" t="inlineStr">
         <is>
@@ -6525,10 +6363,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B86" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B86" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C86" s="20" t="inlineStr">
         <is>
@@ -6581,10 +6417,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B87" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B87" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C87" s="20" t="inlineStr">
         <is>
@@ -6637,10 +6471,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B88" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B88" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C88" s="20" t="inlineStr">
         <is>
@@ -6693,10 +6525,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B89" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B89" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C89" s="20" t="inlineStr">
         <is>
@@ -6749,10 +6579,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B90" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B90" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C90" s="20" t="inlineStr">
         <is>
@@ -6805,10 +6633,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B91" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B91" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C91" s="20" t="inlineStr">
         <is>
@@ -6861,10 +6687,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B92" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B92" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C92" s="20" t="inlineStr">
         <is>
@@ -6917,10 +6741,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B93" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B93" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C93" s="20" t="inlineStr">
         <is>
@@ -6973,10 +6795,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B94" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B94" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C94" s="20" t="inlineStr">
         <is>
@@ -7029,10 +6849,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B95" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B95" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C95" s="20" t="inlineStr">
         <is>
@@ -7085,10 +6903,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B96" s="20" t="inlineStr">
-        <is>
-          <t>10934493</t>
-        </is>
+      <c r="B96" s="20" t="n">
+        <v>10934493</v>
       </c>
       <c r="C96" s="20" t="inlineStr">
         <is>
@@ -7141,10 +6957,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B97" s="20" t="inlineStr">
-        <is>
-          <t>10934493</t>
-        </is>
+      <c r="B97" s="20" t="n">
+        <v>10934493</v>
       </c>
       <c r="C97" s="20" t="inlineStr">
         <is>
@@ -7197,10 +7011,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B98" s="20" t="inlineStr">
-        <is>
-          <t>10934493</t>
-        </is>
+      <c r="B98" s="20" t="n">
+        <v>10934493</v>
       </c>
       <c r="C98" s="20" t="inlineStr">
         <is>
@@ -7253,10 +7065,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B99" s="20" t="inlineStr">
-        <is>
-          <t>10938912</t>
-        </is>
+      <c r="B99" s="20" t="n">
+        <v>10938912</v>
       </c>
       <c r="C99" s="20" t="inlineStr">
         <is>
@@ -7309,10 +7119,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B100" s="20" t="inlineStr">
-        <is>
-          <t>10938912</t>
-        </is>
+      <c r="B100" s="20" t="n">
+        <v>10938912</v>
       </c>
       <c r="C100" s="20" t="inlineStr">
         <is>
@@ -7365,10 +7173,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B101" s="20" t="inlineStr">
-        <is>
-          <t>10938912</t>
-        </is>
+      <c r="B101" s="20" t="n">
+        <v>10938912</v>
       </c>
       <c r="C101" s="20" t="inlineStr">
         <is>
@@ -7421,10 +7227,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B102" s="20" t="inlineStr">
-        <is>
-          <t>10938913</t>
-        </is>
+      <c r="B102" s="20" t="n">
+        <v>10938913</v>
       </c>
       <c r="C102" s="20" t="inlineStr">
         <is>
@@ -7477,10 +7281,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B103" s="20" t="inlineStr">
-        <is>
-          <t>10938913</t>
-        </is>
+      <c r="B103" s="20" t="n">
+        <v>10938913</v>
       </c>
       <c r="C103" s="20" t="inlineStr">
         <is>
@@ -7533,10 +7335,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B104" s="20" t="inlineStr">
-        <is>
-          <t>10938913</t>
-        </is>
+      <c r="B104" s="20" t="n">
+        <v>10938913</v>
       </c>
       <c r="C104" s="20" t="inlineStr">
         <is>
@@ -7589,10 +7389,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B105" s="20" t="inlineStr">
-        <is>
-          <t>10938914</t>
-        </is>
+      <c r="B105" s="20" t="n">
+        <v>10938914</v>
       </c>
       <c r="C105" s="20" t="inlineStr">
         <is>
@@ -7645,10 +7443,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B106" s="20" t="inlineStr">
-        <is>
-          <t>10938914</t>
-        </is>
+      <c r="B106" s="20" t="n">
+        <v>10938914</v>
       </c>
       <c r="C106" s="20" t="inlineStr">
         <is>
@@ -7701,10 +7497,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B107" s="20" t="inlineStr">
-        <is>
-          <t>10938914</t>
-        </is>
+      <c r="B107" s="20" t="n">
+        <v>10938914</v>
       </c>
       <c r="C107" s="20" t="inlineStr">
         <is>
@@ -7757,10 +7551,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B108" s="20" t="inlineStr">
-        <is>
-          <t>10938915</t>
-        </is>
+      <c r="B108" s="20" t="n">
+        <v>10938915</v>
       </c>
       <c r="C108" s="20" t="inlineStr">
         <is>
@@ -7813,10 +7605,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B109" s="20" t="inlineStr">
-        <is>
-          <t>10938915</t>
-        </is>
+      <c r="B109" s="20" t="n">
+        <v>10938915</v>
       </c>
       <c r="C109" s="20" t="inlineStr">
         <is>
@@ -7869,10 +7659,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B110" s="20" t="inlineStr">
-        <is>
-          <t>10938915</t>
-        </is>
+      <c r="B110" s="20" t="n">
+        <v>10938915</v>
       </c>
       <c r="C110" s="20" t="inlineStr">
         <is>
@@ -7925,10 +7713,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B111" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B111" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C111" s="20" t="inlineStr">
         <is>
@@ -7981,10 +7767,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B112" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B112" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C112" s="20" t="inlineStr">
         <is>
@@ -8037,10 +7821,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B113" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B113" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C113" s="20" t="inlineStr">
         <is>
@@ -8093,10 +7875,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B114" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B114" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C114" s="20" t="inlineStr">
         <is>
@@ -8149,10 +7929,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B115" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B115" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C115" s="20" t="inlineStr">
         <is>
@@ -8205,10 +7983,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B116" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B116" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C116" s="20" t="inlineStr">
         <is>
@@ -8261,10 +8037,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B117" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B117" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C117" s="20" t="inlineStr">
         <is>
@@ -8317,10 +8091,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B118" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B118" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C118" s="20" t="inlineStr">
         <is>
@@ -8373,10 +8145,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B119" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B119" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C119" s="20" t="inlineStr">
         <is>
@@ -8429,10 +8199,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B120" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B120" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C120" s="20" t="inlineStr">
         <is>
@@ -8485,10 +8253,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B121" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B121" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C121" s="20" t="inlineStr">
         <is>
@@ -8541,10 +8307,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B122" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B122" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C122" s="20" t="inlineStr">
         <is>
@@ -8597,10 +8361,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B123" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B123" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C123" s="20" t="inlineStr">
         <is>
@@ -8653,10 +8415,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B124" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B124" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C124" s="20" t="inlineStr">
         <is>
@@ -8709,10 +8469,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B125" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B125" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C125" s="20" t="inlineStr">
         <is>
@@ -8765,10 +8523,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B126" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B126" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C126" s="20" t="inlineStr">
         <is>
@@ -8821,10 +8577,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B127" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B127" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C127" s="20" t="inlineStr">
         <is>
@@ -8877,10 +8631,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B128" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B128" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C128" s="20" t="inlineStr">
         <is>
@@ -9019,10 +8771,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>10483607</t>
-        </is>
+      <c r="B5" s="20" t="n">
+        <v>10483607</v>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
@@ -9058,10 +8808,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>10483608</t>
-        </is>
+      <c r="B6" s="20" t="n">
+        <v>10483608</v>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
@@ -9097,10 +8845,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>10521085</t>
-        </is>
+      <c r="B7" s="20" t="n">
+        <v>10521085</v>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
@@ -9136,10 +8882,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>10532818</t>
-        </is>
+      <c r="B8" s="20" t="n">
+        <v>10532818</v>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
@@ -9175,10 +8919,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>10532819</t>
-        </is>
+      <c r="B9" s="20" t="n">
+        <v>10532819</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -9214,10 +8956,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>10615602</t>
-        </is>
+      <c r="B10" s="20" t="n">
+        <v>10615602</v>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
@@ -9253,10 +8993,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>10615603</t>
-        </is>
+      <c r="B11" s="20" t="n">
+        <v>10615603</v>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
@@ -9292,10 +9030,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>10697191</t>
-        </is>
+      <c r="B12" s="20" t="n">
+        <v>10697191</v>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
@@ -9331,10 +9067,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>10711455</t>
-        </is>
+      <c r="B13" s="20" t="n">
+        <v>10711455</v>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
@@ -9370,10 +9104,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>10755051</t>
-        </is>
+      <c r="B14" s="20" t="n">
+        <v>10755051</v>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
@@ -9409,10 +9141,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>10787565</t>
-        </is>
+      <c r="B15" s="20" t="n">
+        <v>10787565</v>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
@@ -9448,10 +9178,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>10810779</t>
-        </is>
+      <c r="B16" s="20" t="n">
+        <v>10810779</v>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
@@ -9487,10 +9215,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>10810780</t>
-        </is>
+      <c r="B17" s="20" t="n">
+        <v>10810780</v>
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
@@ -9526,10 +9252,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>10810782</t>
-        </is>
+      <c r="B18" s="20" t="n">
+        <v>10810782</v>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
@@ -9565,10 +9289,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>10838413</t>
-        </is>
+      <c r="B19" s="20" t="n">
+        <v>10838413</v>
       </c>
       <c r="C19" s="20" t="inlineStr">
         <is>
@@ -9604,10 +9326,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>10838414</t>
-        </is>
+      <c r="B20" s="20" t="n">
+        <v>10838414</v>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
@@ -9643,10 +9363,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>10842437</t>
-        </is>
+      <c r="B21" s="20" t="n">
+        <v>10842437</v>
       </c>
       <c r="C21" s="20" t="inlineStr">
         <is>
@@ -9682,10 +9400,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
-        <is>
-          <t>10864669</t>
-        </is>
+      <c r="B22" s="20" t="n">
+        <v>10864669</v>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
@@ -9721,10 +9437,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>10864670</t>
-        </is>
+      <c r="B23" s="20" t="n">
+        <v>10864670</v>
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
@@ -9760,10 +9474,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
-        <is>
-          <t>10866366</t>
-        </is>
+      <c r="B24" s="20" t="n">
+        <v>10866366</v>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
@@ -9799,10 +9511,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>10908314</t>
-        </is>
+      <c r="B25" s="20" t="n">
+        <v>10908314</v>
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
@@ -9838,10 +9548,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>10908315</t>
-        </is>
+      <c r="B26" s="20" t="n">
+        <v>10908315</v>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
@@ -9877,10 +9585,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
-        <is>
-          <t>10908316</t>
-        </is>
+      <c r="B27" s="20" t="n">
+        <v>10908316</v>
       </c>
       <c r="C27" s="20" t="inlineStr">
         <is>
@@ -9916,10 +9622,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
-        <is>
-          <t>10934493</t>
-        </is>
+      <c r="B28" s="20" t="n">
+        <v>10934493</v>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
@@ -9955,10 +9659,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
-        <is>
-          <t>10935004</t>
-        </is>
+      <c r="B29" s="20" t="n">
+        <v>10935004</v>
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
@@ -9994,10 +9696,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
-        <is>
-          <t>10937405</t>
-        </is>
+      <c r="B30" s="20" t="n">
+        <v>10937405</v>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
@@ -10033,10 +9733,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
-        <is>
-          <t>10938912</t>
-        </is>
+      <c r="B31" s="20" t="n">
+        <v>10938912</v>
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
@@ -10072,10 +9770,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
-        <is>
-          <t>10938913</t>
-        </is>
+      <c r="B32" s="20" t="n">
+        <v>10938913</v>
       </c>
       <c r="C32" s="20" t="inlineStr">
         <is>
@@ -10111,10 +9807,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
-        <is>
-          <t>10938914</t>
-        </is>
+      <c r="B33" s="20" t="n">
+        <v>10938914</v>
       </c>
       <c r="C33" s="20" t="inlineStr">
         <is>
@@ -10150,10 +9844,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
-        <is>
-          <t>10938915</t>
-        </is>
+      <c r="B34" s="20" t="n">
+        <v>10938915</v>
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
@@ -10189,10 +9881,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
-        <is>
-          <t>10938916</t>
-        </is>
+      <c r="B35" s="20" t="n">
+        <v>10938916</v>
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
@@ -10228,10 +9918,8 @@
           <t>Patch</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
-        <is>
-          <t>10938917</t>
-        </is>
+      <c r="B36" s="20" t="n">
+        <v>10938917</v>
       </c>
       <c r="C36" s="20" t="inlineStr">
         <is>
@@ -10267,10 +9955,8 @@
           <t>Core</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
-        <is>
-          <t>10969386</t>
-        </is>
+      <c r="B37" s="20" t="n">
+        <v>10969386</v>
       </c>
       <c r="C37" s="20" t="inlineStr">
         <is>

</xml_diff>